<commit_message>
ingesta: snapshot 2026-09-20 18:10 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-09-20/Temp-max-septiembre-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-09-20/Temp-max-septiembre-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6BDC14F-0F4F-47DF-9335-73BF4C1FFB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D2DD9C3-DF48-4101-8964-906846D3987D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9477,7 +9477,9 @@
       <c r="V5" s="63">
         <v>31.9</v>
       </c>
-      <c r="W5" s="63"/>
+      <c r="W5" s="63">
+        <v>32.1</v>
+      </c>
       <c r="X5" s="63"/>
       <c r="Y5" s="63"/>
       <c r="Z5" s="63"/>
@@ -9492,7 +9494,7 @@
       <c r="AI5" s="63"/>
       <c r="AJ5" s="36">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>31.9</v>
+        <v>32.1</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9510,11 +9512,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>31.80555555555555</v>
+        <v>31.821052631578944</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>0.96841143530798846</v>
+        <v>0.98390851133138213</v>
       </c>
       <c r="AQ5" s="20"/>
     </row>
@@ -9586,7 +9588,9 @@
       <c r="V6" s="63">
         <v>32.799999999999997</v>
       </c>
-      <c r="W6" s="63"/>
+      <c r="W6" s="63">
+        <v>32.6</v>
+      </c>
       <c r="X6" s="63"/>
       <c r="Y6" s="63"/>
       <c r="Z6" s="63"/>
@@ -9601,7 +9605,7 @@
       <c r="AI6" s="63"/>
       <c r="AJ6" s="36">
         <f t="shared" ref="AJ6:AJ48" si="1">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>32.799999999999997</v>
+        <v>32.6</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="2">+MAX($E6:$AI6)</f>
@@ -9619,11 +9623,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="4">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>31.994444444444444</v>
+        <v>32.026315789473685</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="5">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>0.78071959917476264</v>
+        <v>0.81259094420400402</v>
       </c>
       <c r="AQ6" s="20"/>
     </row>
@@ -9695,7 +9699,9 @@
       <c r="V7" s="63">
         <v>35.6</v>
       </c>
-      <c r="W7" s="63"/>
+      <c r="W7" s="63">
+        <v>34.9</v>
+      </c>
       <c r="X7" s="63"/>
       <c r="Y7" s="67"/>
       <c r="Z7" s="63"/>
@@ -9710,7 +9716,7 @@
       <c r="AI7" s="63"/>
       <c r="AJ7" s="36">
         <f t="shared" si="1"/>
-        <v>35.6</v>
+        <v>34.9</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="2"/>
@@ -9728,11 +9734,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="4"/>
-        <v>34.872222222222227</v>
+        <v>34.873684210526314</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="5"/>
-        <v>1.9833420908593382</v>
+        <v>1.9848040791634247</v>
       </c>
       <c r="AQ7" s="20"/>
     </row>
@@ -9804,7 +9810,9 @@
       <c r="V8" s="63">
         <v>33.700000000000003</v>
       </c>
-      <c r="W8" s="63"/>
+      <c r="W8" s="63">
+        <v>33.4</v>
+      </c>
       <c r="X8" s="63"/>
       <c r="Y8" s="63"/>
       <c r="Z8" s="63"/>
@@ -9819,7 +9827,7 @@
       <c r="AI8" s="63"/>
       <c r="AJ8" s="36">
         <f t="shared" si="1"/>
-        <v>33.700000000000003</v>
+        <v>33.4</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="2"/>
@@ -9837,11 +9845,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="4"/>
-        <v>34.272222222222226</v>
+        <v>34.226315789473688</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="5"/>
-        <v>2.2056911084687627</v>
+        <v>2.1597846757202248</v>
       </c>
       <c r="AQ8" s="20"/>
     </row>
@@ -9913,7 +9921,9 @@
       <c r="V9" s="63">
         <v>38.799999999999997</v>
       </c>
-      <c r="W9" s="63"/>
+      <c r="W9" s="63">
+        <v>37</v>
+      </c>
       <c r="X9" s="63"/>
       <c r="Y9" s="63"/>
       <c r="Z9" s="63"/>
@@ -9928,7 +9938,7 @@
       <c r="AI9" s="63"/>
       <c r="AJ9" s="36">
         <f t="shared" si="1"/>
-        <v>38.799999999999997</v>
+        <v>37</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="2"/>
@@ -9946,11 +9956,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="4"/>
-        <v>35.516666666666666</v>
+        <v>35.594736842105263</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="5"/>
-        <v>2.207668965517243</v>
+        <v>2.2857391409558403</v>
       </c>
       <c r="AQ9" s="20"/>
     </row>
@@ -10022,7 +10032,9 @@
       <c r="V10" s="63">
         <v>39.799999999999997</v>
       </c>
-      <c r="W10" s="63"/>
+      <c r="W10" s="63">
+        <v>35.4</v>
+      </c>
       <c r="X10" s="63"/>
       <c r="Y10" s="63"/>
       <c r="Z10" s="63"/>
@@ -10037,7 +10049,7 @@
       <c r="AI10" s="63"/>
       <c r="AJ10" s="36">
         <f t="shared" si="1"/>
-        <v>39.799999999999997</v>
+        <v>35.4</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="2"/>
@@ -10055,11 +10067,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="4"/>
-        <v>36.972222222222214</v>
+        <v>36.889473684210522</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="5"/>
-        <v>3.2123100079996547</v>
+        <v>3.1295614699879621</v>
       </c>
       <c r="AQ10" s="20"/>
     </row>
@@ -10131,7 +10143,9 @@
       <c r="V11" s="63">
         <v>40.6</v>
       </c>
-      <c r="W11" s="63"/>
+      <c r="W11" s="63">
+        <v>35.6</v>
+      </c>
       <c r="X11" s="63"/>
       <c r="Y11" s="63"/>
       <c r="Z11" s="63"/>
@@ -10146,7 +10160,7 @@
       <c r="AI11" s="63"/>
       <c r="AJ11" s="36">
         <f t="shared" si="1"/>
-        <v>40.6</v>
+        <v>35.6</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="2"/>
@@ -10164,11 +10178,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="4"/>
-        <v>38.155555555555551</v>
+        <v>38.021052631578947</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="5"/>
-        <v>4.1433905940802447</v>
+        <v>4.0088876701036398</v>
       </c>
       <c r="AQ11" s="20"/>
     </row>
@@ -10240,7 +10254,9 @@
       <c r="V12" s="63">
         <v>35.4</v>
       </c>
-      <c r="W12" s="63"/>
+      <c r="W12" s="63">
+        <v>28.6</v>
+      </c>
       <c r="X12" s="63"/>
       <c r="Y12" s="63"/>
       <c r="Z12" s="63"/>
@@ -10255,7 +10271,7 @@
       <c r="AI12" s="63"/>
       <c r="AJ12" s="36">
         <f t="shared" si="1"/>
-        <v>35.4</v>
+        <v>28.6</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="2"/>
@@ -10273,11 +10289,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="4"/>
-        <v>34.044444444444444</v>
+        <v>33.757894736842104</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="5"/>
-        <v>2.5918512904719755</v>
+        <v>2.3053015828696353</v>
       </c>
       <c r="AQ12" s="20"/>
     </row>
@@ -10349,7 +10365,9 @@
       <c r="V13" s="63">
         <v>36.6</v>
       </c>
-      <c r="W13" s="63"/>
+      <c r="W13" s="63">
+        <v>31.2</v>
+      </c>
       <c r="X13" s="63"/>
       <c r="Y13" s="63"/>
       <c r="Z13" s="63"/>
@@ -10364,7 +10382,7 @@
       <c r="AI13" s="63"/>
       <c r="AJ13" s="36">
         <f t="shared" si="1"/>
-        <v>36.6</v>
+        <v>31.2</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="2"/>
@@ -10382,11 +10400,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="4"/>
-        <v>34.711111111111116</v>
+        <v>34.526315789473692</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="5"/>
-        <v>2.5113295019157178</v>
+        <v>2.3265341802782942</v>
       </c>
       <c r="AQ13" s="20"/>
     </row>
@@ -10458,7 +10476,9 @@
       <c r="V14" s="63">
         <v>35.200000000000003</v>
       </c>
-      <c r="W14" s="63"/>
+      <c r="W14" s="63">
+        <v>29.6</v>
+      </c>
       <c r="X14" s="63"/>
       <c r="Y14" s="63"/>
       <c r="Z14" s="63"/>
@@ -10473,7 +10493,7 @@
       <c r="AI14" s="63"/>
       <c r="AJ14" s="36">
         <f t="shared" si="1"/>
-        <v>35.200000000000003</v>
+        <v>29.6</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="2"/>
@@ -10491,11 +10511,11 @@
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="4"/>
-        <v>34.288888888888884</v>
+        <v>34.042105263157893</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="5"/>
-        <v>1.7276510078809224</v>
+        <v>1.4808673821499312</v>
       </c>
       <c r="AQ14" s="20"/>
     </row>
@@ -10567,7 +10587,9 @@
       <c r="V15" s="63">
         <v>31.1</v>
       </c>
-      <c r="W15" s="63"/>
+      <c r="W15" s="63">
+        <v>33.6</v>
+      </c>
       <c r="X15" s="63"/>
       <c r="Y15" s="63"/>
       <c r="Z15" s="63"/>
@@ -10582,7 +10604,7 @@
       <c r="AI15" s="63"/>
       <c r="AJ15" s="36">
         <f t="shared" si="1"/>
-        <v>31.1</v>
+        <v>33.6</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="2"/>
@@ -10600,11 +10622,11 @@
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="4"/>
-        <v>31.894444444444446</v>
+        <v>31.984210526315792</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="5"/>
-        <v>-2.3999726327314619E-2</v>
+        <v>6.5766355544031541E-2</v>
       </c>
       <c r="AQ15" s="20"/>
     </row>
@@ -10725,7 +10747,9 @@
       <c r="V17" s="63">
         <v>37.200000000000003</v>
       </c>
-      <c r="W17" s="63"/>
+      <c r="W17" s="63">
+        <v>30</v>
+      </c>
       <c r="X17" s="63"/>
       <c r="Y17" s="63"/>
       <c r="Z17" s="63"/>
@@ -10740,7 +10764,7 @@
       <c r="AI17" s="63"/>
       <c r="AJ17" s="36">
         <f t="shared" si="1"/>
-        <v>37.200000000000003</v>
+        <v>30</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="2"/>
@@ -10758,11 +10782,11 @@
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>35.188888888888897</v>
+        <v>34.915789473684214</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>3.1608865107676039</v>
+        <v>2.8877870955629206</v>
       </c>
       <c r="AQ17" s="20"/>
     </row>
@@ -10834,7 +10858,9 @@
       <c r="V18" s="63">
         <v>28.4</v>
       </c>
-      <c r="W18" s="63"/>
+      <c r="W18" s="63">
+        <v>26.8</v>
+      </c>
       <c r="X18" s="63"/>
       <c r="Y18" s="63"/>
       <c r="Z18" s="63"/>
@@ -10849,7 +10875,7 @@
       <c r="AI18" s="63"/>
       <c r="AJ18" s="36">
         <f t="shared" si="1"/>
-        <v>28.4</v>
+        <v>26.8</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="2"/>
@@ -10867,11 +10893,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="6">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>29.01111111111112</v>
+        <v>28.894736842105271</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="5"/>
-        <v>2.7654975579975591</v>
+        <v>2.64912328899171</v>
       </c>
       <c r="AQ18" s="20"/>
     </row>
@@ -10943,7 +10969,9 @@
       <c r="V19" s="63">
         <v>37.6</v>
       </c>
-      <c r="W19" s="63"/>
+      <c r="W19" s="63">
+        <v>36.299999999999997</v>
+      </c>
       <c r="X19" s="63"/>
       <c r="Y19" s="63"/>
       <c r="Z19" s="63"/>
@@ -10958,7 +10986,7 @@
       <c r="AI19" s="63"/>
       <c r="AJ19" s="36">
         <f t="shared" si="1"/>
-        <v>37.6</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="2"/>
@@ -10976,11 +11004,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="6"/>
-        <v>36.088888888888881</v>
+        <v>36.099999999999994</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="5"/>
-        <v>1.726352969348639</v>
+        <v>1.7374640804597519</v>
       </c>
       <c r="AQ19" s="20"/>
     </row>
@@ -11052,7 +11080,9 @@
       <c r="V20" s="63">
         <v>32.700000000000003</v>
       </c>
-      <c r="W20" s="63"/>
+      <c r="W20" s="63">
+        <v>28.1</v>
+      </c>
       <c r="X20" s="63"/>
       <c r="Y20" s="63"/>
       <c r="Z20" s="63"/>
@@ -11067,7 +11097,7 @@
       <c r="AI20" s="63"/>
       <c r="AJ20" s="36">
         <f t="shared" si="1"/>
-        <v>32.700000000000003</v>
+        <v>28.1</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="2"/>
@@ -11085,11 +11115,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="6"/>
-        <v>30.761111111111113</v>
+        <v>30.621052631578952</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="5"/>
-        <v>2.620893541324584</v>
+        <v>2.4808350617924226</v>
       </c>
       <c r="AQ20" s="20"/>
     </row>
@@ -11161,7 +11191,9 @@
       <c r="V21" s="63">
         <v>25.6</v>
       </c>
-      <c r="W21" s="63"/>
+      <c r="W21" s="63">
+        <v>23.4</v>
+      </c>
       <c r="X21" s="63"/>
       <c r="Y21" s="63"/>
       <c r="Z21" s="63"/>
@@ -11176,7 +11208,7 @@
       <c r="AI21" s="63"/>
       <c r="AJ21" s="36">
         <f t="shared" si="1"/>
-        <v>25.6</v>
+        <v>23.4</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="2"/>
@@ -11194,11 +11226,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="6"/>
-        <v>24.57222222222223</v>
+        <v>24.51052631578948</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="5"/>
-        <v>2.0077870260272306</v>
+        <v>1.946091119594481</v>
       </c>
       <c r="AQ21" s="20"/>
     </row>
@@ -11336,7 +11368,9 @@
       <c r="V23" s="63">
         <v>31.4</v>
       </c>
-      <c r="W23" s="63"/>
+      <c r="W23" s="63">
+        <v>29</v>
+      </c>
       <c r="X23" s="63"/>
       <c r="Y23" s="63"/>
       <c r="Z23" s="63"/>
@@ -11351,7 +11385,7 @@
       <c r="AI23" s="63"/>
       <c r="AJ23" s="36">
         <f t="shared" si="1"/>
-        <v>31.4</v>
+        <v>29</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="2"/>
@@ -11369,11 +11403,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="6"/>
-        <v>29.722222222222221</v>
+        <v>29.684210526315791</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="5"/>
-        <v>2.6822531682876516</v>
+        <v>2.6442414723812213</v>
       </c>
       <c r="AQ23" s="20"/>
     </row>
@@ -11445,7 +11479,9 @@
       <c r="V24" s="63">
         <v>33.799999999999997</v>
       </c>
-      <c r="W24" s="63"/>
+      <c r="W24" s="63">
+        <v>32.700000000000003</v>
+      </c>
       <c r="X24" s="63"/>
       <c r="Y24" s="63"/>
       <c r="Z24" s="63"/>
@@ -11460,7 +11496,7 @@
       <c r="AI24" s="63"/>
       <c r="AJ24" s="36">
         <f t="shared" si="1"/>
-        <v>33.799999999999997</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="2"/>
@@ -11478,11 +11514,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="6"/>
-        <v>31.299999999999997</v>
+        <v>31.373684210526317</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="5"/>
-        <v>3.0803922641853667</v>
+        <v>3.1540764747116867</v>
       </c>
       <c r="AQ24" s="20"/>
     </row>
@@ -11554,7 +11590,9 @@
       <c r="V25" s="63">
         <v>36.1</v>
       </c>
-      <c r="W25" s="63"/>
+      <c r="W25" s="63">
+        <v>34.700000000000003</v>
+      </c>
       <c r="X25" s="63"/>
       <c r="Y25" s="63"/>
       <c r="Z25" s="63"/>
@@ -11569,7 +11607,7 @@
       <c r="AI25" s="63"/>
       <c r="AJ25" s="36">
         <f t="shared" si="1"/>
-        <v>36.1</v>
+        <v>34.700000000000003</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="2"/>
@@ -11587,11 +11625,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="6"/>
-        <v>34.277777777777786</v>
+        <v>34.300000000000011</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="5"/>
-        <v>3.4412889983579653</v>
+        <v>3.463511220580191</v>
       </c>
       <c r="AQ25" s="20"/>
     </row>
@@ -11663,7 +11701,9 @@
       <c r="V26" s="63">
         <v>19.3</v>
       </c>
-      <c r="W26" s="63"/>
+      <c r="W26" s="63">
+        <v>20.7</v>
+      </c>
       <c r="X26" s="63"/>
       <c r="Y26" s="63"/>
       <c r="Z26" s="63"/>
@@ -11678,7 +11718,7 @@
       <c r="AI26" s="63"/>
       <c r="AJ26" s="36">
         <f t="shared" si="1"/>
-        <v>19.3</v>
+        <v>20.7</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="2"/>
@@ -11696,11 +11736,11 @@
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="6"/>
-        <v>20.161111111111111</v>
+        <v>20.189473684210526</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="5"/>
-        <v>0.95608343886195257</v>
+        <v>0.98444601196136716</v>
       </c>
       <c r="AQ26" s="20"/>
     </row>
@@ -11772,7 +11812,9 @@
       <c r="V27" s="63">
         <v>21.2</v>
       </c>
-      <c r="W27" s="63"/>
+      <c r="W27" s="63">
+        <v>19.2</v>
+      </c>
       <c r="X27" s="63"/>
       <c r="Y27" s="63"/>
       <c r="Z27" s="63"/>
@@ -11787,7 +11829,7 @@
       <c r="AI27" s="63"/>
       <c r="AJ27" s="36">
         <f t="shared" si="1"/>
-        <v>21.2</v>
+        <v>19.2</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="2"/>
@@ -11805,11 +11847,11 @@
       </c>
       <c r="AO27" s="23">
         <f t="shared" si="6"/>
-        <v>20.622222222222224</v>
+        <v>20.547368421052635</v>
       </c>
       <c r="AP27" s="23">
         <f t="shared" si="5"/>
-        <v>2.528232074438975</v>
+        <v>2.4533782732693865</v>
       </c>
       <c r="AQ27" s="20"/>
     </row>
@@ -11881,7 +11923,9 @@
       <c r="V28" s="63">
         <v>35.299999999999997</v>
       </c>
-      <c r="W28" s="63"/>
+      <c r="W28" s="63">
+        <v>34.9</v>
+      </c>
       <c r="X28" s="63"/>
       <c r="Y28" s="63"/>
       <c r="Z28" s="63"/>
@@ -11896,7 +11940,7 @@
       <c r="AI28" s="63"/>
       <c r="AJ28" s="36">
         <f t="shared" si="1"/>
-        <v>35.299999999999997</v>
+        <v>34.9</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="2"/>
@@ -11914,11 +11958,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="6"/>
-        <v>33.655555555555551</v>
+        <v>33.721052631578942</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="5"/>
-        <v>3.01510711510711</v>
+        <v>3.0806041911305009</v>
       </c>
       <c r="AQ28" s="20"/>
     </row>
@@ -12054,7 +12098,9 @@
       <c r="V30" s="63">
         <v>38</v>
       </c>
-      <c r="W30" s="63"/>
+      <c r="W30" s="63">
+        <v>36.700000000000003</v>
+      </c>
       <c r="X30" s="63"/>
       <c r="Y30" s="63"/>
       <c r="Z30" s="63"/>
@@ -12069,7 +12115,7 @@
       <c r="AI30" s="63"/>
       <c r="AJ30" s="36">
         <f t="shared" si="1"/>
-        <v>38</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="2"/>
@@ -12087,11 +12133,11 @@
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="6"/>
-        <v>36.783333333333339</v>
+        <v>36.778947368421065</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="5"/>
-        <v>1.8714444444444496</v>
+        <v>1.8670584795321759</v>
       </c>
       <c r="AQ30" s="20"/>
     </row>
@@ -12163,7 +12209,9 @@
       <c r="V31" s="63">
         <v>28.3</v>
       </c>
-      <c r="W31" s="63"/>
+      <c r="W31" s="63">
+        <v>27</v>
+      </c>
       <c r="X31" s="63"/>
       <c r="Y31" s="63"/>
       <c r="Z31" s="63"/>
@@ -12178,7 +12226,7 @@
       <c r="AI31" s="63"/>
       <c r="AJ31" s="36">
         <f t="shared" si="1"/>
-        <v>28.3</v>
+        <v>27</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="2"/>
@@ -12196,11 +12244,11 @@
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="6"/>
-        <v>28.083333333333332</v>
+        <v>28.026315789473685</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="5"/>
-        <v>2.1009459637997132</v>
+        <v>2.043928419940066</v>
       </c>
       <c r="AQ31" s="20"/>
     </row>
@@ -12272,7 +12320,9 @@
       <c r="V32" s="63">
         <v>17.2</v>
       </c>
-      <c r="W32" s="63"/>
+      <c r="W32" s="63">
+        <v>16.600000000000001</v>
+      </c>
       <c r="X32" s="63"/>
       <c r="Y32" s="63"/>
       <c r="Z32" s="63"/>
@@ -12287,7 +12337,7 @@
       <c r="AI32" s="63"/>
       <c r="AJ32" s="36">
         <f t="shared" si="1"/>
-        <v>17.2</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="2"/>
@@ -12305,11 +12355,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="6"/>
-        <v>18.555555555555557</v>
+        <v>18.452631578947372</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="5"/>
-        <v>1.2193322533640867</v>
+        <v>1.1164082767559016</v>
       </c>
       <c r="AQ32" s="20"/>
     </row>
@@ -12381,7 +12431,9 @@
       <c r="V33" s="63">
         <v>15.8</v>
       </c>
-      <c r="W33" s="63"/>
+      <c r="W33" s="63">
+        <v>14.6</v>
+      </c>
       <c r="X33" s="63"/>
       <c r="Y33" s="63"/>
       <c r="Z33" s="63"/>
@@ -12396,7 +12448,7 @@
       <c r="AI33" s="63"/>
       <c r="AJ33" s="36">
         <f t="shared" si="1"/>
-        <v>15.8</v>
+        <v>14.6</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="2"/>
@@ -12414,11 +12466,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="6"/>
-        <v>16.600000000000005</v>
+        <v>16.494736842105269</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="5"/>
-        <v>0.66969029374202549</v>
+        <v>0.56442713584728921</v>
       </c>
       <c r="AQ33" s="20"/>
       <c r="AT33" s="15"/>
@@ -12542,7 +12594,9 @@
       <c r="V35" s="63">
         <v>31.2</v>
       </c>
-      <c r="W35" s="63"/>
+      <c r="W35" s="63">
+        <v>32.799999999999997</v>
+      </c>
       <c r="X35" s="63"/>
       <c r="Y35" s="63"/>
       <c r="Z35" s="63"/>
@@ -12557,7 +12611,7 @@
       <c r="AI35" s="63"/>
       <c r="AJ35" s="36">
         <f t="shared" si="1"/>
-        <v>31.2</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="2"/>
@@ -12575,11 +12629,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>31.899999999999995</v>
+        <v>31.947368421052627</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="5"/>
-        <v>0.95288615216201578</v>
+        <v>1.0002545732146473</v>
       </c>
       <c r="AQ35" s="20"/>
       <c r="AT35" s="15"/>
@@ -12770,7 +12824,9 @@
       <c r="V38" s="63">
         <v>33.700000000000003</v>
       </c>
-      <c r="W38" s="63"/>
+      <c r="W38" s="63">
+        <v>30.1</v>
+      </c>
       <c r="X38" s="63"/>
       <c r="Y38" s="63"/>
       <c r="Z38" s="63"/>
@@ -12785,7 +12841,7 @@
       <c r="AI38" s="63"/>
       <c r="AJ38" s="36">
         <f t="shared" si="1"/>
-        <v>33.700000000000003</v>
+        <v>30.1</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="2"/>
@@ -12803,11 +12859,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>32.894444444444446</v>
+        <v>32.747368421052634</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="5"/>
-        <v>1.2229729976281654</v>
+        <v>1.075896974236354</v>
       </c>
       <c r="AQ38" s="20"/>
       <c r="AT38" s="15"/>
@@ -12880,7 +12936,9 @@
       <c r="V39" s="63">
         <v>30</v>
       </c>
-      <c r="W39" s="63"/>
+      <c r="W39" s="63">
+        <v>31.4</v>
+      </c>
       <c r="X39" s="63"/>
       <c r="Y39" s="63"/>
       <c r="Z39" s="63"/>
@@ -12895,7 +12953,7 @@
       <c r="AI39" s="63"/>
       <c r="AJ39" s="36">
         <f t="shared" si="1"/>
-        <v>30</v>
+        <v>31.4</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="2"/>
@@ -12913,11 +12971,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="8">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>33.538888888888884</v>
+        <v>33.426315789473676</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="5"/>
-        <v>0.8540256308627221</v>
+        <v>0.74145253144751422</v>
       </c>
       <c r="AQ39" s="20"/>
       <c r="AT39" s="15"/>
@@ -12990,7 +13048,9 @@
       <c r="V40" s="63">
         <v>28</v>
       </c>
-      <c r="W40" s="63"/>
+      <c r="W40" s="63">
+        <v>31.7</v>
+      </c>
       <c r="X40" s="63"/>
       <c r="Y40" s="63"/>
       <c r="Z40" s="63"/>
@@ -13005,7 +13065,7 @@
       <c r="AI40" s="63"/>
       <c r="AJ40" s="36">
         <f t="shared" si="1"/>
-        <v>28</v>
+        <v>31.7</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="2"/>
@@ -13023,11 +13083,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="8"/>
-        <v>31.711111111111116</v>
+        <v>31.71052631578948</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="5"/>
-        <v>0.91212917350848599</v>
+        <v>0.91154437818684997</v>
       </c>
       <c r="AQ40" s="20"/>
       <c r="AT40" s="15"/>
@@ -13100,7 +13160,9 @@
       <c r="V41" s="63">
         <v>32.200000000000003</v>
       </c>
-      <c r="W41" s="63"/>
+      <c r="W41" s="63">
+        <v>31.4</v>
+      </c>
       <c r="X41" s="63"/>
       <c r="Y41" s="63"/>
       <c r="Z41" s="63"/>
@@ -13115,7 +13177,7 @@
       <c r="AI41" s="63"/>
       <c r="AJ41" s="36">
         <f t="shared" si="1"/>
-        <v>32.200000000000003</v>
+        <v>31.4</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="2"/>
@@ -13133,11 +13195,11 @@
       </c>
       <c r="AO41" s="23">
         <f t="shared" si="8"/>
-        <v>31.533333333333342</v>
+        <v>31.526315789473689</v>
       </c>
       <c r="AP41" s="23">
         <f t="shared" si="5"/>
-        <v>0.91781773399015165</v>
+        <v>0.91080019013049807</v>
       </c>
       <c r="AQ41" s="20"/>
       <c r="AT41" s="15"/>
@@ -13278,7 +13340,9 @@
       <c r="V43" s="63">
         <v>32.200000000000003</v>
       </c>
-      <c r="W43" s="63"/>
+      <c r="W43" s="63">
+        <v>34</v>
+      </c>
       <c r="X43" s="63"/>
       <c r="Y43" s="63"/>
       <c r="Z43" s="63"/>
@@ -13293,7 +13357,7 @@
       <c r="AI43" s="63"/>
       <c r="AJ43" s="36">
         <f t="shared" si="1"/>
-        <v>32.200000000000003</v>
+        <v>34</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="2"/>
@@ -13311,11 +13375,11 @@
       </c>
       <c r="AO43" s="23">
         <f t="shared" si="8"/>
-        <v>32.433333333333337</v>
+        <v>32.515789473684215</v>
       </c>
       <c r="AP43" s="23">
         <f t="shared" si="5"/>
-        <v>0.44202926956377553</v>
+        <v>0.52448540991465364</v>
       </c>
       <c r="AQ43" s="20"/>
       <c r="AT43" s="15"/>
@@ -13388,7 +13452,9 @@
       <c r="V44" s="29">
         <v>33</v>
       </c>
-      <c r="W44" s="29"/>
+      <c r="W44" s="29">
+        <v>32</v>
+      </c>
       <c r="X44" s="29"/>
       <c r="Y44" s="29"/>
       <c r="Z44" s="29"/>
@@ -13403,7 +13469,7 @@
       <c r="AI44" s="63"/>
       <c r="AJ44" s="36">
         <f t="shared" si="1"/>
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="2"/>
@@ -13421,11 +13487,11 @@
       </c>
       <c r="AO44" s="23">
         <f t="shared" si="8"/>
-        <v>31.611111111111111</v>
+        <v>31.631578947368421</v>
       </c>
       <c r="AP44" s="23">
         <f t="shared" si="5"/>
-        <v>0.51117354902795142</v>
+        <v>0.53164138528526195</v>
       </c>
       <c r="AQ44" s="20"/>
       <c r="AT44" s="15"/>
@@ -13498,7 +13564,9 @@
       <c r="V45" s="63">
         <v>31.8</v>
       </c>
-      <c r="W45" s="63"/>
+      <c r="W45" s="63">
+        <v>32.200000000000003</v>
+      </c>
       <c r="X45" s="63"/>
       <c r="Y45" s="63"/>
       <c r="Z45" s="63"/>
@@ -13513,7 +13581,7 @@
       <c r="AI45" s="63"/>
       <c r="AJ45" s="36">
         <f t="shared" si="1"/>
-        <v>31.8</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="2"/>
@@ -13531,11 +13599,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="8"/>
-        <v>32.24444444444444</v>
+        <v>32.242105263157896</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="5"/>
-        <v>0.76621398197368862</v>
+        <v>0.76387480068714453</v>
       </c>
       <c r="AQ45" s="20"/>
       <c r="AT45" s="15"/>
@@ -13740,7 +13808,9 @@
       <c r="V48" s="63">
         <v>32.6</v>
       </c>
-      <c r="W48" s="63"/>
+      <c r="W48" s="63">
+        <v>30.4</v>
+      </c>
       <c r="X48" s="63"/>
       <c r="Y48" s="63"/>
       <c r="Z48" s="63"/>
@@ -13755,7 +13825,7 @@
       <c r="AI48" s="63"/>
       <c r="AJ48" s="36">
         <f t="shared" si="1"/>
-        <v>32.6</v>
+        <v>30.4</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="2"/>
@@ -13773,11 +13843,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="8"/>
-        <v>31.950000000000003</v>
+        <v>31.868421052631579</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="5"/>
-        <v>-3.8443854995566795E-2</v>
+        <v>-0.12002280236399088</v>
       </c>
       <c r="AQ48" s="20"/>
     </row>
@@ -26833,12 +26903,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -26848,6 +26912,12 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>